<commit_message>
Document large-cap+midcap universe robustness check in assumptions
A separate exploration (not part of this repo) re-tuned and
walk-forward-validated the same approach on a large-cap + midcap-only
universe (200 stocks, no smallcap) and found it outperforms this
submission's full 300-stock strategy on both return and risk-adjusted
return, at the cost of a deeper drawdown. Kept the full 300-stock
universe here since the competition brief requires it - added a
transparency note explaining the finding to export_excel.py's
Model_Logic_Assumptions sheet and README.md rather than switching
universes.
</commit_message>
<xml_diff>
--- a/citadel_submission.xlsx
+++ b/citadel_submission.xlsx
@@ -674,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1222,6 +1222,18 @@
       <c r="B56" s="8" t="inlineStr">
         <is>
           <t>NIFTY50, NIFTY500_TMI</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Universe robustness check</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>This submission uses the full specified 300-stock universe (Nifty 100 + Midcap 100 + Smallcap 100) as required. As a separate robustness check, we also re-tuned and backtested a large-cap + midcap-only universe (Nifty 50 + Nifty Next 50 + Nifty Midcap 100, 200 stocks, no smallcap) with independently walk-forward-validated weights (momentum 55% / low-vol 10% / 52-week-high 25% / liquidity 10%). It outperformed the full-universe strategy on both return and risk-adjusted return (test-period Sharpe 1.70 vs. this submission's, at a cost of a deeper max drawdown), suggesting smallcap noise dilutes signal quality for this factor set - but we kept the full 300-stock universe here to comply with the competition's stated requirement.</t>
         </is>
       </c>
     </row>
@@ -66687,10 +66699,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -66884,6 +66896,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Universe robustness check</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>This submission uses the full specified 300-stock universe (Nifty 100 + Midcap 100 + Smallcap 100) as required. As a separate robustness check, we also re-tuned and backtested a large-cap + midcap-only universe (Nifty 50 + Nifty Next 50 + Nifty Midcap 100, 200 stocks, no smallcap) with independently walk-forward-validated weights (momentum 55% / low-vol 10% / 52-week-high 25% / liquidity 10%). It outperformed the full-universe strategy on both return and risk-adjusted return (test-period Sharpe 1.70 vs. this submission's, at a cost of a deeper max drawdown), suggesting smallcap noise dilutes signal quality for this factor set - but we kept the full 300-stock universe here to comply with the competition's stated requirement.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>